<commit_message>
add realdata based uk data files
</commit_message>
<xml_diff>
--- a/01_data/uk/qgis_export_uk.xlsx
+++ b/01_data/uk/qgis_export_uk.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MINJI\NETWORK RELIABILITY\QGIS\8.UK\json\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Minji Kang\Documents\GitHub\railnet_opt\01_data\uk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB4C2B49-6D25-478A-9B43-C3DFD069F781}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09BE54AC-290B-4D9D-9BC8-CF6C8C62FF97}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NODE" sheetId="1" r:id="rId1"/>

</xml_diff>